<commit_message>
Fix visitsQuery date range filter fallback for summary and time slicer
</commit_message>
<xml_diff>
--- a/orders.xlsx
+++ b/orders.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>python scripts\pulpoplus_extract_visits.py "path\to\your\downloaded_file.xls"</t>
   </si>
@@ -45,6 +45,24 @@
   </si>
   <si>
     <t>Team Hierarchy Changes</t>
+  </si>
+  <si>
+    <t>node check_visits.js "Rep Name" 2026-07-01</t>
+  </si>
+  <si>
+    <t>rep data</t>
+  </si>
+  <si>
+    <t>python pulpoplus_rebuild_summary.py "E:\crm extractor\Periods\recent\July 2026 - Eagles 1.xlsx "</t>
+  </si>
+  <si>
+    <t>git add .</t>
+  </si>
+  <si>
+    <t>git commit -m "Fix deployment"</t>
+  </si>
+  <si>
+    <t>git push origin main</t>
   </si>
 </sst>
 </file>
@@ -1204,8 +1222,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="1"/>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="123.555555555556" customWidth="1"/>
     <col min="2" max="2" width="43.6666666666667" customWidth="1"/>
@@ -1235,6 +1253,34 @@
         <v>5</v>
       </c>
     </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>